<commit_message>
tests, randomness check alg for shelling
</commit_message>
<xml_diff>
--- a/examples/benchmark_results/gmm_discretization_results_test_2025-06-18_1.xlsx
+++ b/examples/benchmark_results/gmm_discretization_results_test_2025-06-18_1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,28 +480,28 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="D2" t="n">
-        <v>1.239227414131165</v>
+        <v>2.276271343231201</v>
       </c>
       <c r="E2" t="n">
-        <v>1.220449328422546</v>
+        <v>2.017783880233765</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1483519077301025</v>
+        <v>2.413547039031982</v>
       </c>
       <c r="G2" t="n">
-        <v>0.03263521194458008</v>
+        <v>0.2587378025054932</v>
       </c>
       <c r="H2" t="n">
         <v>97</v>
       </c>
       <c r="I2" t="n">
-        <v>45</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3">
@@ -509,28 +509,28 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>14</v>
+        <v>91</v>
       </c>
       <c r="D3" t="n">
-        <v>1.057926416397095</v>
+        <v>0.2641818225383759</v>
       </c>
       <c r="E3" t="n">
-        <v>1.055729985237122</v>
+        <v>0.9648607969284058</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1899039745330811</v>
+        <v>1.749530792236328</v>
       </c>
       <c r="G3" t="n">
-        <v>0.03384828567504883</v>
+        <v>0.135624885559082</v>
       </c>
       <c r="H3" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I3" t="n">
-        <v>59</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4">
@@ -541,25 +541,25 @@
         <v>8</v>
       </c>
       <c r="C4" t="n">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="D4" t="n">
-        <v>2.301715850830078</v>
+        <v>2.012369632720947</v>
       </c>
       <c r="E4" t="n">
-        <v>1.999168992042542</v>
+        <v>1.795571088790894</v>
       </c>
       <c r="F4" t="n">
-        <v>1.477953195571899</v>
+        <v>0.2318112850189209</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1948087215423584</v>
+        <v>0.06235980987548828</v>
       </c>
       <c r="H4" t="n">
         <v>97</v>
       </c>
       <c r="I4" t="n">
-        <v>47</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5">
@@ -567,28 +567,28 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>81</v>
+        <v>37</v>
       </c>
       <c r="D5" t="n">
-        <v>0.6050302982330322</v>
+        <v>1.037206888198853</v>
       </c>
       <c r="E5" t="n">
-        <v>1.222379922866821</v>
+        <v>1.466828107833862</v>
       </c>
       <c r="F5" t="n">
-        <v>2.061585903167725</v>
+        <v>0.5892238616943359</v>
       </c>
       <c r="G5" t="n">
-        <v>0.155081033706665</v>
+        <v>0.09356331825256348</v>
       </c>
       <c r="H5" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I5" t="n">
-        <v>81</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6">
@@ -596,144 +596,173 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2.440292596817017</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.674623012542725</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.1744639873504639</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.04894900321960449</v>
+      </c>
+      <c r="H6" t="n">
         <v>97</v>
       </c>
-      <c r="D6" t="n">
-        <v>1.058426856994629</v>
-      </c>
-      <c r="E6" t="n">
-        <v>1.41524076461792</v>
-      </c>
-      <c r="F6" t="n">
-        <v>3.562422037124634</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.2280499935150146</v>
-      </c>
-      <c r="H6" t="n">
-        <v>82</v>
-      </c>
       <c r="I6" t="n">
-        <v>97</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>58</v>
+        <v>92</v>
       </c>
       <c r="D7" t="n">
-        <v>0.6732411980628967</v>
+        <v>1.715517640113831</v>
       </c>
       <c r="E7" t="n">
-        <v>1.209251642227173</v>
+        <v>1.742815613746643</v>
       </c>
       <c r="F7" t="n">
-        <v>1.017589092254639</v>
+        <v>4.453652143478394</v>
       </c>
       <c r="G7" t="n">
-        <v>0.112529993057251</v>
+        <v>0.3813169002532959</v>
       </c>
       <c r="H7" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I7" t="n">
-        <v>58</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C8" t="n">
-        <v>62</v>
+        <v>9</v>
       </c>
       <c r="D8" t="n">
-        <v>0.6738578677177429</v>
+        <v>1.256444573402405</v>
       </c>
       <c r="E8" t="n">
-        <v>1.27300488948822</v>
+        <v>1.03722357749939</v>
       </c>
       <c r="F8" t="n">
-        <v>1.152599096298218</v>
+        <v>0.09250998497009277</v>
       </c>
       <c r="G8" t="n">
-        <v>0.1164929866790771</v>
+        <v>0.02820301055908203</v>
       </c>
       <c r="H8" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I8" t="n">
-        <v>62</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C9" t="n">
-        <v>22</v>
+        <v>83</v>
       </c>
       <c r="D9" t="n">
-        <v>1.544310927391052</v>
+        <v>0.2585581839084625</v>
       </c>
       <c r="E9" t="n">
-        <v>1.638338923454285</v>
+        <v>0.9754124283790588</v>
       </c>
       <c r="F9" t="n">
-        <v>0.3976380825042725</v>
+        <v>1.444708108901978</v>
       </c>
       <c r="G9" t="n">
-        <v>0.07448816299438477</v>
+        <v>0.1244618892669678</v>
       </c>
       <c r="H9" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I9" t="n">
-        <v>22</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" t="n">
+        <v>99</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.2802687585353851</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1.011287093162537</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2.098603010177612</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.1495749950408936</v>
+      </c>
+      <c r="H10" t="n">
+        <v>101</v>
+      </c>
+      <c r="I10" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
         <v>10</v>
       </c>
-      <c r="B10" t="n">
-        <v>8</v>
-      </c>
-      <c r="C10" t="n">
-        <v>75</v>
-      </c>
-      <c r="D10" t="n">
-        <v>2.435090065002441</v>
-      </c>
-      <c r="E10" t="n">
-        <v>2.02686071395874</v>
-      </c>
-      <c r="F10" t="n">
-        <v>3.322917222976685</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.3255007266998291</v>
-      </c>
-      <c r="H10" t="n">
+      <c r="B11" t="n">
+        <v>7</v>
+      </c>
+      <c r="C11" t="n">
+        <v>88</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1.943400621414185</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1.87008810043335</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4.804750204086304</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.5541248321533203</v>
+      </c>
+      <c r="H11" t="n">
         <v>97</v>
       </c>
-      <c r="I10" t="n">
-        <v>75</v>
+      <c r="I11" t="n">
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>